<commit_message>
MACD scan results 2026-08-20
</commit_message>
<xml_diff>
--- a/results/2026-08-20.xlsx
+++ b/results/2026-08-20.xlsx
@@ -904,13 +904,13 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>BBY</t>
+          <t>BCPC</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>CUBE</t>
+          <t>CVCO</t>
         </is>
       </c>
     </row>
@@ -919,13 +919,13 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>BCRX</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>CVSA</t>
         </is>
       </c>
     </row>
@@ -934,13 +934,13 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>BCRX</t>
+          <t>BHP</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>DAR</t>
         </is>
       </c>
     </row>
@@ -949,13 +949,13 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>BHP</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>DAR</t>
+          <t>DASH</t>
         </is>
       </c>
     </row>
@@ -964,13 +964,13 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>BMY</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>DC</t>
         </is>
       </c>
     </row>
@@ -979,13 +979,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>BMY</t>
+          <t>BP</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>DC</t>
+          <t>DINO</t>
         </is>
       </c>
     </row>
@@ -994,13 +994,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>BP</t>
+          <t>BTE</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>DINO</t>
+          <t>DRH</t>
         </is>
       </c>
     </row>
@@ -1009,13 +1009,13 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>BTE</t>
+          <t>CADL</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>DRH</t>
+          <t>ECL</t>
         </is>
       </c>
     </row>
@@ -1024,13 +1024,13 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CADL</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ECL</t>
+          <t>EGO</t>
         </is>
       </c>
     </row>
@@ -1039,13 +1039,13 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CBRE</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>EGO</t>
+          <t>ELS</t>
         </is>
       </c>
     </row>
@@ -1054,13 +1054,13 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CBRE</t>
+          <t>CGON</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ELS</t>
+          <t>EMBJ</t>
         </is>
       </c>
     </row>
@@ -1069,13 +1069,13 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>CGON</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>EMBJ</t>
+          <t>EQIX</t>
         </is>
       </c>
     </row>
@@ -1084,13 +1084,13 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CLH</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>ET</t>
         </is>
       </c>
     </row>
@@ -1099,13 +1099,13 @@
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CLH</t>
+          <t>CLYM</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ET</t>
+          <t>EW</t>
         </is>
       </c>
     </row>
@@ -1114,13 +1114,13 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CLYM</t>
+          <t>CMBT</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>EW</t>
+          <t>EXK</t>
         </is>
       </c>
     </row>
@@ -1129,13 +1129,13 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CMBT</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>EXK</t>
+          <t>EXPD</t>
         </is>
       </c>
     </row>
@@ -1144,13 +1144,13 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>CORT</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>EXPD</t>
+          <t>FIGS</t>
         </is>
       </c>
     </row>
@@ -1159,13 +1159,13 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>CRGY</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>FCFS</t>
+          <t>FOX</t>
         </is>
       </c>
     </row>
@@ -1174,13 +1174,13 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CRGY</t>
+          <t>CRON</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>FIGS</t>
+          <t>FOXA</t>
         </is>
       </c>
     </row>
@@ -1189,13 +1189,13 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>CRON</t>
+          <t>CVE</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>FOX</t>
+          <t>GKOS</t>
         </is>
       </c>
     </row>
@@ -1204,13 +1204,13 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CVE</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>FOXA</t>
+          <t>GLNG</t>
         </is>
       </c>
     </row>
@@ -1219,13 +1219,13 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>CWK</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>GKOS</t>
+          <t>GOLD</t>
         </is>
       </c>
     </row>
@@ -1234,13 +1234,13 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CWK</t>
+          <t>DHT</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>GLNG</t>
+          <t>GPCR</t>
         </is>
       </c>
     </row>
@@ -1249,13 +1249,13 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>DHT</t>
+          <t>DJCO</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>GOLD</t>
+          <t>GTE</t>
         </is>
       </c>
     </row>
@@ -1264,13 +1264,13 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>DJCO</t>
+          <t>DNLI</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>GPCR</t>
+          <t>HASI</t>
         </is>
       </c>
     </row>
@@ -1279,13 +1279,13 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>DNLI</t>
+          <t>DSX</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>GTE</t>
+          <t>HBM</t>
         </is>
       </c>
     </row>
@@ -1294,13 +1294,13 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>DSX</t>
+          <t>DUOT</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>HASI</t>
+          <t>HLN</t>
         </is>
       </c>
     </row>
@@ -1309,13 +1309,13 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>DUOT</t>
+          <t>DVN</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>HBM</t>
+          <t>HLX</t>
         </is>
       </c>
     </row>
@@ -1324,13 +1324,13 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>DVN</t>
+          <t>DX</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>HLN</t>
+          <t>HP</t>
         </is>
       </c>
     </row>
@@ -1339,13 +1339,13 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>DX</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>HLX</t>
+          <t>HZO</t>
         </is>
       </c>
     </row>
@@ -1354,13 +1354,13 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>ECO</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>IAUX</t>
         </is>
       </c>
     </row>
@@ -1369,13 +1369,13 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ECO</t>
+          <t>EFC</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>HZO</t>
+          <t>ICUI</t>
         </is>
       </c>
     </row>
@@ -1384,13 +1384,13 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>EFC</t>
+          <t>EGY</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>IAUX</t>
+          <t>IHS</t>
         </is>
       </c>
     </row>
@@ -1399,13 +1399,13 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>EGY</t>
+          <t>EOG</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ICUI</t>
+          <t>ILMN</t>
         </is>
       </c>
     </row>
@@ -1414,13 +1414,13 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>EOG</t>
+          <t>EQNR</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>IHS</t>
+          <t>IMAX</t>
         </is>
       </c>
     </row>
@@ -1429,13 +1429,13 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>EQNR</t>
+          <t>ETON</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>ITIC</t>
         </is>
       </c>
     </row>
@@ -1444,13 +1444,13 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ETON</t>
+          <t>EWTX</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
-          <t>IMAX</t>
+          <t>LOAR</t>
         </is>
       </c>
     </row>
@@ -1459,13 +1459,13 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>EWTX</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ITIC</t>
+          <t>LTC</t>
         </is>
       </c>
     </row>
@@ -1474,13 +1474,13 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>LOAR</t>
+          <t>LXRX</t>
         </is>
       </c>
     </row>
@@ -1489,13 +1489,13 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>FLR</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
-          <t>LTC</t>
+          <t>MATX</t>
         </is>
       </c>
     </row>
@@ -1504,13 +1504,13 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>FLR</t>
+          <t>FNV</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
-          <t>LXRX</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
@@ -1519,13 +1519,13 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>FNV</t>
+          <t>FRHC</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
-          <t>MATX</t>
+          <t>MGA</t>
         </is>
       </c>
     </row>
@@ -1534,13 +1534,13 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>FRHC</t>
+          <t>FRNM</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>MPC</t>
         </is>
       </c>
     </row>
@@ -1549,13 +1549,13 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>FRNM</t>
+          <t>FRO</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
-          <t>MGA</t>
+          <t>MRAM</t>
         </is>
       </c>
     </row>
@@ -1564,13 +1564,13 @@
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
-          <t>FRO</t>
+          <t>FSM</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
-          <t>MPC</t>
+          <t>MRX</t>
         </is>
       </c>
     </row>
@@ -1579,13 +1579,13 @@
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
-          <t>FSM</t>
+          <t>FWONK</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
-          <t>MRAM</t>
+          <t>MSI</t>
         </is>
       </c>
     </row>
@@ -1594,13 +1594,13 @@
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
-          <t>FWONK</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
-          <t>MRX</t>
+          <t>MU</t>
         </is>
       </c>
     </row>
@@ -1609,13 +1609,13 @@
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>NSC</t>
         </is>
       </c>
     </row>
@@ -1624,13 +1624,13 @@
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>NTRA</t>
         </is>
       </c>
     </row>
@@ -1639,13 +1639,13 @@
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>HAE</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
-          <t>NSC</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
@@ -1654,13 +1654,13 @@
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
-          <t>HAE</t>
+          <t>HAFN</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>OMC</t>
         </is>
       </c>
     </row>
@@ -1669,13 +1669,13 @@
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
-          <t>HAFN</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>PAA</t>
         </is>
       </c>
     </row>
@@ -1684,13 +1684,13 @@
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>HCC</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
-          <t>OMC</t>
+          <t>PBR</t>
         </is>
       </c>
     </row>
@@ -1699,13 +1699,13 @@
       <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
-          <t>HCC</t>
+          <t>HMY</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>PDM</t>
         </is>
       </c>
     </row>
@@ -1714,13 +1714,13 @@
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr">
         <is>
-          <t>HMY</t>
+          <t>HRMY</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
-          <t>PBR</t>
+          <t>PEN</t>
         </is>
       </c>
     </row>
@@ -1729,13 +1729,13 @@
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
-          <t>HRMY</t>
+          <t>HTGC</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
-          <t>PDM</t>
+          <t>PHM</t>
         </is>
       </c>
     </row>
@@ -1744,13 +1744,13 @@
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
-          <t>HTGC</t>
+          <t>IAG</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
-          <t>PEN</t>
+          <t>PM</t>
         </is>
       </c>
     </row>
@@ -1759,13 +1759,13 @@
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
-          <t>IAG</t>
+          <t>IBRX</t>
         </is>
       </c>
       <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr">
         <is>
-          <t>PHM</t>
+          <t>PRAX</t>
         </is>
       </c>
     </row>
@@ -1774,13 +1774,13 @@
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>IDYA</t>
         </is>
       </c>
       <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr">
         <is>
-          <t>PM</t>
+          <t>PRCH</t>
         </is>
       </c>
     </row>
@@ -1789,13 +1789,13 @@
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr">
         <is>
-          <t>IDYA</t>
+          <t>IMMX</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
-          <t>PRAX</t>
+          <t>PSX</t>
         </is>
       </c>
     </row>
@@ -1804,13 +1804,13 @@
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
-          <t>IMMX</t>
+          <t>IMNM</t>
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>QSR</t>
         </is>
       </c>
     </row>
@@ -1819,13 +1819,13 @@
       <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
         <is>
-          <t>IMNM</t>
+          <t>IMO</t>
         </is>
       </c>
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr">
         <is>
-          <t>PSX</t>
+          <t>REAL</t>
         </is>
       </c>
     </row>
@@ -1834,13 +1834,13 @@
       <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr">
         <is>
-          <t>IMO</t>
+          <t>IMVT</t>
         </is>
       </c>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
         <is>
-          <t>QSR</t>
+          <t>RIG</t>
         </is>
       </c>
     </row>
@@ -1849,13 +1849,13 @@
       <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
-          <t>IMVT</t>
+          <t>INBX</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
-          <t>RIG</t>
+          <t>RYAM</t>
         </is>
       </c>
     </row>
@@ -1864,13 +1864,13 @@
       <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr">
         <is>
-          <t>INBX</t>
+          <t>INCY</t>
         </is>
       </c>
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
-          <t>RYAM</t>
+          <t>SA</t>
         </is>
       </c>
     </row>
@@ -1879,13 +1879,13 @@
       <c r="B91" t="inlineStr"/>
       <c r="C91" t="inlineStr">
         <is>
-          <t>INCY</t>
+          <t>INSW</t>
         </is>
       </c>
       <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>SAIC</t>
         </is>
       </c>
     </row>
@@ -1894,13 +1894,13 @@
       <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr">
         <is>
-          <t>INSW</t>
+          <t>JLL</t>
         </is>
       </c>
       <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>SBRA</t>
         </is>
       </c>
     </row>
@@ -1909,13 +1909,13 @@
       <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr">
         <is>
-          <t>JLL</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
         <is>
-          <t>SBRA</t>
+          <t>SGMT</t>
         </is>
       </c>
     </row>
@@ -1924,13 +1924,13 @@
       <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr">
         <is>
-          <t>JNJ</t>
+          <t>KNTK</t>
         </is>
       </c>
       <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr">
         <is>
-          <t>SGMT</t>
+          <t>SKM</t>
         </is>
       </c>
     </row>
@@ -1939,13 +1939,13 @@
       <c r="B95" t="inlineStr"/>
       <c r="C95" t="inlineStr">
         <is>
-          <t>KNTK</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
-          <t>SJM</t>
+          <t>SLAB</t>
         </is>
       </c>
     </row>
@@ -1954,13 +1954,13 @@
       <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>KYMR</t>
         </is>
       </c>
       <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
-          <t>SKM</t>
+          <t>SLB</t>
         </is>
       </c>
     </row>
@@ -1969,13 +1969,13 @@
       <c r="B97" t="inlineStr"/>
       <c r="C97" t="inlineStr">
         <is>
-          <t>KYMR</t>
+          <t>LAUR</t>
         </is>
       </c>
       <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr">
         <is>
-          <t>SLAB</t>
+          <t>SOLV</t>
         </is>
       </c>
     </row>
@@ -1984,13 +1984,13 @@
       <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>STLN</t>
         </is>
       </c>
     </row>
@@ -1999,13 +1999,13 @@
       <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>LFST</t>
         </is>
       </c>
       <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr">
         <is>
-          <t>SOLV</t>
+          <t>STNG</t>
         </is>
       </c>
     </row>
@@ -2014,13 +2014,13 @@
       <c r="B100" t="inlineStr"/>
       <c r="C100" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>LIVN</t>
         </is>
       </c>
       <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>SVM</t>
         </is>
       </c>
     </row>
@@ -2029,13 +2029,13 @@
       <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
-          <t>STNG</t>
+          <t>SWX</t>
         </is>
       </c>
     </row>
@@ -2044,13 +2044,13 @@
       <c r="B102" t="inlineStr"/>
       <c r="C102" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>LNG</t>
         </is>
       </c>
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr">
         <is>
-          <t>SVM</t>
+          <t>SXT</t>
         </is>
       </c>
     </row>
@@ -2059,13 +2059,13 @@
       <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr">
         <is>
-          <t>LNG</t>
+          <t>LPG</t>
         </is>
       </c>
       <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr">
         <is>
-          <t>SWX</t>
+          <t>TDW</t>
         </is>
       </c>
     </row>
@@ -2074,13 +2074,13 @@
       <c r="B104" t="inlineStr"/>
       <c r="C104" t="inlineStr">
         <is>
-          <t>LPG</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr">
         <is>
-          <t>SXT</t>
+          <t>TEVA</t>
         </is>
       </c>
     </row>
@@ -2089,13 +2089,13 @@
       <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>MCO</t>
         </is>
       </c>
       <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr">
         <is>
-          <t>TDW</t>
+          <t>TH</t>
         </is>
       </c>
     </row>
@@ -2104,13 +2104,13 @@
       <c r="B106" t="inlineStr"/>
       <c r="C106" t="inlineStr">
         <is>
-          <t>MCO</t>
+          <t>MDT</t>
         </is>
       </c>
       <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr">
         <is>
-          <t>TEVA</t>
+          <t>THM</t>
         </is>
       </c>
     </row>
@@ -2119,13 +2119,13 @@
       <c r="B107" t="inlineStr"/>
       <c r="C107" t="inlineStr">
         <is>
-          <t>MDT</t>
+          <t>MGTX</t>
         </is>
       </c>
       <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>TPG</t>
         </is>
       </c>
     </row>
@@ -2134,13 +2134,13 @@
       <c r="B108" t="inlineStr"/>
       <c r="C108" t="inlineStr">
         <is>
-          <t>MGTX</t>
+          <t>MHO</t>
         </is>
       </c>
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr">
         <is>
-          <t>THM</t>
+          <t>U</t>
         </is>
       </c>
     </row>
@@ -2149,13 +2149,13 @@
       <c r="B109" t="inlineStr"/>
       <c r="C109" t="inlineStr">
         <is>
-          <t>MHO</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>UL</t>
         </is>
       </c>
     </row>
@@ -2164,13 +2164,13 @@
       <c r="B110" t="inlineStr"/>
       <c r="C110" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>UNP</t>
         </is>
       </c>
     </row>
@@ -2179,13 +2179,13 @@
       <c r="B111" t="inlineStr"/>
       <c r="C111" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr">
         <is>
-          <t>UL</t>
+          <t>URGN</t>
         </is>
       </c>
     </row>
@@ -2194,13 +2194,13 @@
       <c r="B112" t="inlineStr"/>
       <c r="C112" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr">
         <is>
-          <t>UNP</t>
+          <t>VAL</t>
         </is>
       </c>
     </row>
@@ -2209,13 +2209,13 @@
       <c r="B113" t="inlineStr"/>
       <c r="C113" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MTDR</t>
         </is>
       </c>
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr">
         <is>
-          <t>URGN</t>
+          <t>VIRT</t>
         </is>
       </c>
     </row>
@@ -2224,13 +2224,13 @@
       <c r="B114" t="inlineStr"/>
       <c r="C114" t="inlineStr">
         <is>
-          <t>MTDR</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr">
         <is>
-          <t>VAL</t>
+          <t>VLO</t>
         </is>
       </c>
     </row>
@@ -2239,13 +2239,13 @@
       <c r="B115" t="inlineStr"/>
       <c r="C115" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
         <is>
-          <t>VIRT</t>
+          <t>W</t>
         </is>
       </c>
     </row>
@@ -2254,13 +2254,13 @@
       <c r="B116" t="inlineStr"/>
       <c r="C116" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>NEM</t>
         </is>
       </c>
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr">
         <is>
-          <t>VLO</t>
+          <t>WELL</t>
         </is>
       </c>
     </row>
@@ -2269,13 +2269,13 @@
       <c r="B117" t="inlineStr"/>
       <c r="C117" t="inlineStr">
         <is>
-          <t>NEM</t>
+          <t>NLY</t>
         </is>
       </c>
       <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>WMS</t>
         </is>
       </c>
     </row>
@@ -2284,13 +2284,13 @@
       <c r="B118" t="inlineStr"/>
       <c r="C118" t="inlineStr">
         <is>
-          <t>NLY</t>
+          <t>NRIX</t>
         </is>
       </c>
       <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr">
         <is>
-          <t>WELL</t>
+          <t>WST</t>
         </is>
       </c>
     </row>
@@ -2299,13 +2299,13 @@
       <c r="B119" t="inlineStr"/>
       <c r="C119" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>NTR</t>
         </is>
       </c>
       <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr">
         <is>
-          <t>WES</t>
+          <t>ZM</t>
         </is>
       </c>
     </row>
@@ -2314,52 +2314,40 @@
       <c r="B120" t="inlineStr"/>
       <c r="C120" t="inlineStr">
         <is>
-          <t>NTR</t>
+          <t>NUVB</t>
         </is>
       </c>
       <c r="D120" t="inlineStr"/>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>WMS</t>
-        </is>
-      </c>
+      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr"/>
       <c r="B121" t="inlineStr"/>
       <c r="C121" t="inlineStr">
         <is>
-          <t>NUVB</t>
+          <t>NVS</t>
         </is>
       </c>
       <c r="D121" t="inlineStr"/>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>WST</t>
-        </is>
-      </c>
+      <c r="E121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr"/>
       <c r="B122" t="inlineStr"/>
       <c r="C122" t="inlineStr">
         <is>
-          <t>NVS</t>
+          <t>NWS</t>
         </is>
       </c>
       <c r="D122" t="inlineStr"/>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>ZM</t>
-        </is>
-      </c>
+      <c r="E122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr"/>
       <c r="B123" t="inlineStr"/>
       <c r="C123" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="D123" t="inlineStr"/>
@@ -2370,7 +2358,7 @@
       <c r="B124" t="inlineStr"/>
       <c r="C124" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>OBE</t>
         </is>
       </c>
       <c r="D124" t="inlineStr"/>
@@ -2381,7 +2369,7 @@
       <c r="B125" t="inlineStr"/>
       <c r="C125" t="inlineStr">
         <is>
-          <t>OBE</t>
+          <t>OCUL</t>
         </is>
       </c>
       <c r="D125" t="inlineStr"/>
@@ -2392,7 +2380,7 @@
       <c r="B126" t="inlineStr"/>
       <c r="C126" t="inlineStr">
         <is>
-          <t>OCUL</t>
+          <t>OKE</t>
         </is>
       </c>
       <c r="D126" t="inlineStr"/>
@@ -2403,7 +2391,7 @@
       <c r="B127" t="inlineStr"/>
       <c r="C127" t="inlineStr">
         <is>
-          <t>OKE</t>
+          <t>OMER</t>
         </is>
       </c>
       <c r="D127" t="inlineStr"/>
@@ -2414,7 +2402,7 @@
       <c r="B128" t="inlineStr"/>
       <c r="C128" t="inlineStr">
         <is>
-          <t>OMER</t>
+          <t>ONC</t>
         </is>
       </c>
       <c r="D128" t="inlineStr"/>
@@ -2425,7 +2413,7 @@
       <c r="B129" t="inlineStr"/>
       <c r="C129" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>ORC</t>
         </is>
       </c>
       <c r="D129" t="inlineStr"/>
@@ -2436,7 +2424,7 @@
       <c r="B130" t="inlineStr"/>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ORC</t>
+          <t>ORIC</t>
         </is>
       </c>
       <c r="D130" t="inlineStr"/>
@@ -2447,7 +2435,7 @@
       <c r="B131" t="inlineStr"/>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ORIC</t>
+          <t>OSCR</t>
         </is>
       </c>
       <c r="D131" t="inlineStr"/>
@@ -2458,7 +2446,7 @@
       <c r="B132" t="inlineStr"/>
       <c r="C132" t="inlineStr">
         <is>
-          <t>OSCR</t>
+          <t>OVID</t>
         </is>
       </c>
       <c r="D132" t="inlineStr"/>
@@ -2469,7 +2457,7 @@
       <c r="B133" t="inlineStr"/>
       <c r="C133" t="inlineStr">
         <is>
-          <t>OVID</t>
+          <t>OVV</t>
         </is>
       </c>
       <c r="D133" t="inlineStr"/>
@@ -2480,7 +2468,7 @@
       <c r="B134" t="inlineStr"/>
       <c r="C134" t="inlineStr">
         <is>
-          <t>OVV</t>
+          <t>OXY</t>
         </is>
       </c>
       <c r="D134" t="inlineStr"/>
@@ -2491,7 +2479,7 @@
       <c r="B135" t="inlineStr"/>
       <c r="C135" t="inlineStr">
         <is>
-          <t>OXY</t>
+          <t>PAGP</t>
         </is>
       </c>
       <c r="D135" t="inlineStr"/>
@@ -2502,7 +2490,7 @@
       <c r="B136" t="inlineStr"/>
       <c r="C136" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>PCG</t>
         </is>
       </c>
       <c r="D136" t="inlineStr"/>
@@ -2513,7 +2501,7 @@
       <c r="B137" t="inlineStr"/>
       <c r="C137" t="inlineStr">
         <is>
-          <t>PCG</t>
+          <t>PCVX</t>
         </is>
       </c>
       <c r="D137" t="inlineStr"/>
@@ -2524,7 +2512,7 @@
       <c r="B138" t="inlineStr"/>
       <c r="C138" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>PHVS</t>
         </is>
       </c>
       <c r="D138" t="inlineStr"/>
@@ -2535,7 +2523,7 @@
       <c r="B139" t="inlineStr"/>
       <c r="C139" t="inlineStr">
         <is>
-          <t>PHVS</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="D139" t="inlineStr"/>
@@ -2546,7 +2534,7 @@
       <c r="B140" t="inlineStr"/>
       <c r="C140" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="D140" t="inlineStr"/>
@@ -2557,7 +2545,7 @@
       <c r="B141" t="inlineStr"/>
       <c r="C141" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>PSNL</t>
         </is>
       </c>
       <c r="D141" t="inlineStr"/>
@@ -2568,7 +2556,7 @@
       <c r="B142" t="inlineStr"/>
       <c r="C142" t="inlineStr">
         <is>
-          <t>PSNL</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="D142" t="inlineStr"/>
@@ -2579,7 +2567,7 @@
       <c r="B143" t="inlineStr"/>
       <c r="C143" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>QURE</t>
         </is>
       </c>
       <c r="D143" t="inlineStr"/>
@@ -2590,7 +2578,7 @@
       <c r="B144" t="inlineStr"/>
       <c r="C144" t="inlineStr">
         <is>
-          <t>QURE</t>
+          <t>RCUS</t>
         </is>
       </c>
       <c r="D144" t="inlineStr"/>
@@ -2601,7 +2589,7 @@
       <c r="B145" t="inlineStr"/>
       <c r="C145" t="inlineStr">
         <is>
-          <t>RCUS</t>
+          <t>RIO</t>
         </is>
       </c>
       <c r="D145" t="inlineStr"/>
@@ -2612,7 +2600,7 @@
       <c r="B146" t="inlineStr"/>
       <c r="C146" t="inlineStr">
         <is>
-          <t>RIO</t>
+          <t>RLAY</t>
         </is>
       </c>
       <c r="D146" t="inlineStr"/>
@@ -2623,7 +2611,7 @@
       <c r="B147" t="inlineStr"/>
       <c r="C147" t="inlineStr">
         <is>
-          <t>RLAY</t>
+          <t>ROIV</t>
         </is>
       </c>
       <c r="D147" t="inlineStr"/>
@@ -2634,7 +2622,7 @@
       <c r="B148" t="inlineStr"/>
       <c r="C148" t="inlineStr">
         <is>
-          <t>ROIV</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="D148" t="inlineStr"/>
@@ -2645,7 +2633,7 @@
       <c r="B149" t="inlineStr"/>
       <c r="C149" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>RSG</t>
         </is>
       </c>
       <c r="D149" t="inlineStr"/>
@@ -2656,7 +2644,7 @@
       <c r="B150" t="inlineStr"/>
       <c r="C150" t="inlineStr">
         <is>
-          <t>RSG</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="D150" t="inlineStr"/>
@@ -2667,7 +2655,7 @@
       <c r="B151" t="inlineStr"/>
       <c r="C151" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>SBLK</t>
         </is>
       </c>
       <c r="D151" t="inlineStr"/>
@@ -2678,7 +2666,7 @@
       <c r="B152" t="inlineStr"/>
       <c r="C152" t="inlineStr">
         <is>
-          <t>SBLK</t>
+          <t>SCCO</t>
         </is>
       </c>
       <c r="D152" t="inlineStr"/>

</xml_diff>